<commit_message>
Excel: título del gráfico con la conclusión
</commit_message>
<xml_diff>
--- a/resultados/rebanada1.xlsx
+++ b/resultados/rebanada1.xlsx
@@ -178,7 +178,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Pérdida con descuento mayor al 20%, por subcategoría (US$)</a:t>
+              <a:t>Binders, Tables y Machines concentran el 72% de la pérdida (US$)</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -627,7 +627,7 @@
           <t>Binders</t>
         </is>
       </c>
-      <c r="B2" s="2" t="n">
+      <c r="B2" s="3" t="n">
         <v>613</v>
       </c>
       <c r="C2" s="3" t="n">
@@ -659,7 +659,7 @@
           <t>Tables</t>
         </is>
       </c>
-      <c r="B3" s="2" t="n">
+      <c r="B3" s="3" t="n">
         <v>176</v>
       </c>
       <c r="C3" s="3" t="n">
@@ -691,7 +691,7 @@
           <t>Machines</t>
         </is>
       </c>
-      <c r="B4" s="2" t="n">
+      <c r="B4" s="3" t="n">
         <v>53</v>
       </c>
       <c r="C4" s="3" t="n">
@@ -723,7 +723,7 @@
           <t>Bookcases</t>
         </is>
       </c>
-      <c r="B5" s="2" t="n">
+      <c r="B5" s="3" t="n">
         <v>70</v>
       </c>
       <c r="C5" s="3" t="n">
@@ -755,7 +755,7 @@
           <t>Appliances</t>
         </is>
       </c>
-      <c r="B6" s="2" t="n">
+      <c r="B6" s="3" t="n">
         <v>67</v>
       </c>
       <c r="C6" s="3" t="n">
@@ -787,7 +787,7 @@
           <t>Chairs</t>
         </is>
       </c>
-      <c r="B7" s="2" t="n">
+      <c r="B7" s="3" t="n">
         <v>158</v>
       </c>
       <c r="C7" s="3" t="n">
@@ -819,7 +819,7 @@
           <t>Phones</t>
         </is>
       </c>
-      <c r="B8" s="2" t="n">
+      <c r="B8" s="3" t="n">
         <v>109</v>
       </c>
       <c r="C8" s="3" t="n">
@@ -851,7 +851,7 @@
           <t>Furnishings</t>
         </is>
       </c>
-      <c r="B9" s="2" t="n">
+      <c r="B9" s="3" t="n">
         <v>138</v>
       </c>
       <c r="C9" s="3" t="n">
@@ -883,7 +883,7 @@
           <t>Copiers</t>
         </is>
       </c>
-      <c r="B10" s="2" t="n">
+      <c r="B10" s="3" t="n">
         <v>9</v>
       </c>
       <c r="C10" s="3" t="n">
@@ -915,7 +915,7 @@
           <t>Total</t>
         </is>
       </c>
-      <c r="B11" s="6">
+      <c r="B11" s="7">
         <f>SUM(B2:B10)</f>
         <v/>
       </c>

</xml_diff>